<commit_message>
Apply FR->PL gold review corrections; apply neutral-possessive convention consistently to controls and FR->PL annotations; regenerate tables
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4iHamavskXUSLfNBvgnUc
</commit_message>
<xml_diff>
--- a/data_fr_pl/gold_review_sheet.xlsx
+++ b/data_fr_pl/gold_review_sheet.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -441,42 +441,28 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>How to review (one row at a time, or in batches of ~28):</t>
+          <t>Gold review sheet (updated 2026-10-22 after the authors' review of the FR-&gt;PL gold).</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1. Meaning: read the original sentence (column B) and the gloss of the gold (column F). Does the gold keep the meaning of the original? Mark OK or Problem.</t>
+          <t>FR-&gt;PL gold: reviewed by the authors; corrections applied (ID2, 5, 21-23, 32, 33, 39, 49-52). PL-&gt;FR (French) gold: not yet reviewed.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2. Gender: does the gold show the gender that the source (column C) shows? For rows with signal N (yellow) the source has no gender; both variants are accepted.</t>
+          <t>For each row: Meaning OK? Gender OK? Comment.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3. Neutral-by-design rows (possessives, imperatives, tu/vous): the convention of the original dataset is kept (feminine possessor).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4. Write any problem in column J. A second AI may be used for hard rows; if so, record it in the comment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>The glosses were written by Claude from the gold; they are a reading aid, not a ground truth. Neither the gold nor the glosses have been checked by a native speaker.</t>
+          <t>Glosses were written by Claude as a reading aid; neither gold nor glosses were checked by a native speaker.</t>
         </is>
       </c>
     </row>
@@ -617,7 +603,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>One pomalowały sobie usta i paznokcie, a one założyły spódnice.</t>
+          <t>One pomalowały sobie usta i paznokcie i założyły spódnice.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -719,7 +705,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>One zdecydowały założyć własną firmę.</t>
+          <t>One zdecydowały się założyć własną firmę.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1303,7 +1289,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Jej książka jest bardzo interesująca.</t>
+          <t>Jej książka jest bardzo interesująca. / Jego książka jest bardzo interesująca.</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1313,7 +1299,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>possessor gender not marked in source; feminine follows the original design</t>
+          <t>possessor gender not marked in source; either form accepted (dataset convention: any 3rd/2nd-person rendering is acceptable)</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr"/>
@@ -1341,7 +1327,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Jej buty są nowe.</t>
+          <t>Jej buty są nowe. / Jego buty są nowe.</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1351,7 +1337,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>as 21</t>
+          <t>possessor gender not marked in source; either form accepted (dataset convention: any 3rd/2nd-person rendering is acceptable)</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr"/>
@@ -1379,7 +1365,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Jej teczka zaginęła wczoraj.</t>
+          <t>Jej teczka zaginęła wczoraj. / Jego teczka zaginęła wczoraj.</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1389,7 +1375,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>as 21</t>
+          <t>possessor gender not marked in source; either form accepted (dataset convention: any 3rd/2nd-person rendering is acceptable)</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr"/>
@@ -1689,7 +1675,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>One zawsze pomagają jedna drugiej.</t>
+          <t>One zawsze pomagają sobie nawzajem.</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -1723,7 +1709,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>One wspierają jedna drugą w pracy.</t>
+          <t>One wspierają się nawzajem w pracy.</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -1939,7 +1925,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Ta ławka tam.</t>
+          <t>Tamta ławka.</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2291,7 +2277,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Ty masz się dobrze.</t>
+          <t>Dobrze się masz.</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -2325,7 +2311,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Wy macie się dobrze.</t>
+          <t>Dobrze się macie.</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
@@ -2359,7 +2345,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Wy jesteście bardzo dobre.</t>
+          <t>Jesteście bardzo dobre.</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -2393,7 +2379,7 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Wy jesteście bardzo dobrzy.</t>
+          <t>Jesteście bardzo dobrzy.</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Review PL->FR (French) gold: no change, notes for IDs 18-21; lock FR<->PL annotations
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4iHamavskXUSLfNBvgnUc
</commit_message>
<xml_diff>
--- a/data_fr_pl/gold_review_sheet.xlsx
+++ b/data_fr_pl/gold_review_sheet.xlsx
@@ -448,7 +448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FR-&gt;PL gold: reviewed by the authors; corrections applied (ID2, 5, 21-23, 32, 33, 39, 49-52). PL-&gt;FR (French) gold: not yet reviewed.</t>
+          <t>FR-&gt;PL gold (Polish): reviewed by the authors, corrections applied (ID2, 5, 21-23, 32, 33, 39, 49-52). PL-&gt;FR gold (French): reviewed by the authors with a second-opinion analysis by another AI; no change needed (notes added to IDs 18-21). No native speaker was involved.</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>possessor gender not marked in French; feminine follows the original design</t>
+          <t>French cannot mark the possessor's gender ('son/ses'); the source (Polish 'Jej') can. Information loss in the target language, not a system error; any 'son/ses' rendering is correct</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>as 18</t>
+          <t>French cannot mark the possessor's gender ('son/ses'); the source (Polish 'Jej') can. Information loss in the target language, not a system error; any 'son/ses' rendering is correct</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>as 18</t>
+          <t>French cannot mark the possessor's gender ('son/ses'); the source (Polish 'Jej') can. Information loss in the target language, not a system error; any 'son/ses' rendering is correct</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>as 18</t>
+          <t>French cannot mark the possessor's gender ('son/ses'); the source (Polish 'Jej') can. Information loss in the target language, not a system error; any 'son/ses' rendering is correct</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr"/>

</xml_diff>